<commit_message>
fix: SPB-8 decimals, editable accounts, broker dropdown, LT default
- SPB-8 Section 03: amounts in thousands with 2 decimals (both
  SPB-8 Excel generator and Данъчна accounts sheet)
- SPB-8 Section 04: quantities with 2 decimal places (numFmt 0.00)
- Foreign accounts: Edit button moves account to editable form
- Broker dropdown: populated from foreignAccounts + brokerInterest
  (works after Excel import, not just file import)
- Default country for manual Revolut accounts: LT (Lithuania)
- Update AGENTS.md and README.md
- Regenerate reference Excel
</commit_message>
<xml_diff>
--- a/samples/Данъчна_2025.xlsx
+++ b/samples/Данъчна_2025.xlsx
@@ -1509,7 +1509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1520,6 +1520,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15829,11 +15830,11 @@
       <c r="G2" s="4">
         <v>44058.25</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="10">
         <v>0</v>
       </c>
-      <c r="I2" s="1">
-        <v>44</v>
+      <c r="I2" s="10">
+        <v>44.06</v>
       </c>
       <c r="J2" s="4">
         <v>86170.4470975</v>
@@ -15861,11 +15862,11 @@
       <c r="G3" s="4">
         <v>5050.9</v>
       </c>
-      <c r="H3" s="1">
-        <v>11</v>
-      </c>
-      <c r="I3" s="1">
-        <v>5</v>
+      <c r="H3" s="10">
+        <v>10.5</v>
+      </c>
+      <c r="I3" s="10">
+        <v>5.05</v>
       </c>
       <c r="J3" s="4">
         <v>9498.75167980769</v>
@@ -15893,11 +15894,11 @@
       <c r="G4" s="4">
         <v>-1887.6</v>
       </c>
-      <c r="H4" s="1">
-        <v>0</v>
-      </c>
-      <c r="I4" s="1">
-        <v>-2</v>
+      <c r="H4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="I4" s="10">
+        <v>-1.89</v>
       </c>
       <c r="J4" s="4">
         <v>-3691.8247079999996</v>
@@ -15925,11 +15926,11 @@
       <c r="G5" s="4">
         <v>6633.54</v>
       </c>
-      <c r="H5" s="1">
-        <v>6</v>
-      </c>
-      <c r="I5" s="1">
-        <v>7</v>
+      <c r="H5" s="10">
+        <v>5.81</v>
+      </c>
+      <c r="I5" s="10">
+        <v>6.63</v>
       </c>
       <c r="J5" s="4">
         <v>12475.073594423076</v>
@@ -15957,11 +15958,11 @@
       <c r="G6" s="4">
         <v>200</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="10">
         <v>0</v>
       </c>
-      <c r="I6" s="1">
-        <v>0</v>
+      <c r="I6" s="10">
+        <v>0.2</v>
       </c>
       <c r="J6" s="4">
         <v>471.28433734939756</v>
@@ -15989,11 +15990,11 @@
       <c r="G7" s="4">
         <v>300</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="10">
         <v>0</v>
       </c>
-      <c r="I7" s="1">
-        <v>0</v>
+      <c r="I7" s="10">
+        <v>0.3</v>
       </c>
       <c r="J7" s="4">
         <v>586.749</v>

</xml_diff>

<commit_message>
fix: SPB-8 decimals, editable accounts, broker dropdown, LT default (#20)
- SPB-8 Section 03: amounts in thousands with 2 decimals (both
  SPB-8 Excel generator and Данъчна accounts sheet)
- SPB-8 Section 04: quantities with 2 decimal places (numFmt 0.00)
- Foreign accounts: Edit button moves account to editable form
- Broker dropdown: populated from foreignAccounts + brokerInterest
  (works after Excel import, not just file import)
- Default country for manual Revolut accounts: LT (Lithuania)
- Update AGENTS.md and README.md
- Regenerate reference Excel
</commit_message>
<xml_diff>
--- a/samples/Данъчна_2025.xlsx
+++ b/samples/Данъчна_2025.xlsx
@@ -1509,7 +1509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1520,6 +1520,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15829,11 +15830,11 @@
       <c r="G2" s="4">
         <v>44058.25</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="10">
         <v>0</v>
       </c>
-      <c r="I2" s="1">
-        <v>44</v>
+      <c r="I2" s="10">
+        <v>44.06</v>
       </c>
       <c r="J2" s="4">
         <v>86170.4470975</v>
@@ -15861,11 +15862,11 @@
       <c r="G3" s="4">
         <v>5050.9</v>
       </c>
-      <c r="H3" s="1">
-        <v>11</v>
-      </c>
-      <c r="I3" s="1">
-        <v>5</v>
+      <c r="H3" s="10">
+        <v>10.5</v>
+      </c>
+      <c r="I3" s="10">
+        <v>5.05</v>
       </c>
       <c r="J3" s="4">
         <v>9498.75167980769</v>
@@ -15893,11 +15894,11 @@
       <c r="G4" s="4">
         <v>-1887.6</v>
       </c>
-      <c r="H4" s="1">
-        <v>0</v>
-      </c>
-      <c r="I4" s="1">
-        <v>-2</v>
+      <c r="H4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="I4" s="10">
+        <v>-1.89</v>
       </c>
       <c r="J4" s="4">
         <v>-3691.8247079999996</v>
@@ -15925,11 +15926,11 @@
       <c r="G5" s="4">
         <v>6633.54</v>
       </c>
-      <c r="H5" s="1">
-        <v>6</v>
-      </c>
-      <c r="I5" s="1">
-        <v>7</v>
+      <c r="H5" s="10">
+        <v>5.81</v>
+      </c>
+      <c r="I5" s="10">
+        <v>6.63</v>
       </c>
       <c r="J5" s="4">
         <v>12475.073594423076</v>
@@ -15957,11 +15958,11 @@
       <c r="G6" s="4">
         <v>200</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="10">
         <v>0</v>
       </c>
-      <c r="I6" s="1">
-        <v>0</v>
+      <c r="I6" s="10">
+        <v>0.2</v>
       </c>
       <c r="J6" s="4">
         <v>471.28433734939756</v>
@@ -15989,11 +15990,11 @@
       <c r="G7" s="4">
         <v>300</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="10">
         <v>0</v>
       </c>
-      <c r="I7" s="1">
-        <v>0</v>
+      <c r="I7" s="10">
+        <v>0.3</v>
       </c>
       <c r="J7" s="4">
         <v>586.749</v>

</xml_diff>